<commit_message>
Major restructure and update of drought analysis project
</commit_message>
<xml_diff>
--- a/temporal_drought/basin_averaged_timeseries/Drought_Summary_Statistics.xlsx
+++ b/temporal_drought/basin_averaged_timeseries/Drought_Summary_Statistics.xlsx
@@ -7,13 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="Summary_Statistics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Correlations_Scale3" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Correlations_All" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">Timescale</t>
   </si>
@@ -39,12 +39,18 @@
     <t xml:space="preserve">Drought_Events_2020_2025</t>
   </si>
   <si>
+    <t xml:space="preserve">Data_Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">01</t>
   </si>
   <si>
     <t xml:space="preserve">SPI</t>
   </si>
   <si>
+    <t xml:space="preserve">Gridded</t>
+  </si>
+  <si>
     <t xml:space="preserve">03</t>
   </si>
   <si>
@@ -55,6 +61,12 @@
   </si>
   <si>
     <t xml:space="preserve">SPEI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSPI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSPEI</t>
   </si>
   <si>
     <t xml:space="preserve">Comparison</t>
@@ -426,13 +438,16 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
         <v>-0.00671772326777806</v>
@@ -452,13 +467,16 @@
       <c r="H2" t="n">
         <v>3</v>
       </c>
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
       </c>
       <c r="C3" t="n">
         <v>-0.00526030218976795</v>
@@ -478,13 +496,16 @@
       <c r="H3" t="n">
         <v>1</v>
       </c>
+      <c r="I3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
         <v>-0.00514941999844803</v>
@@ -504,13 +525,16 @@
       <c r="H4" t="n">
         <v>2</v>
       </c>
+      <c r="I4" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>0.00567652694896697</v>
@@ -530,13 +554,16 @@
       <c r="H5" t="n">
         <v>1</v>
       </c>
+      <c r="I5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
         <v>0.000721012300872929</v>
@@ -556,13 +583,16 @@
       <c r="H6" t="n">
         <v>6</v>
       </c>
+      <c r="I6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" t="n">
         <v>-0.0015255361931585</v>
@@ -582,13 +612,16 @@
       <c r="H7" t="n">
         <v>1</v>
       </c>
+      <c r="I7" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" t="n">
         <v>0.00106774424215219</v>
@@ -608,13 +641,16 @@
       <c r="H8" t="n">
         <v>2</v>
       </c>
+      <c r="I8" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n">
         <v>0.00483153946603219</v>
@@ -633,6 +669,67 @@
       </c>
       <c r="H9" t="n">
         <v>1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-0.00000221975582685843</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.610740244835506</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-1.338</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3.184</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-0.00000998890122086604</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.005</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.415864853728681</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.931</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.271</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -648,10 +745,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>